<commit_message>
Aggregate: focus on 4 ticket params with league avg/min/max + rank + grade
Rework the club aggregate to the parameters the analytical note needs:
average ticket price (regular season), online sales share, free-ticket share,
and actual attendance deviation (protocol vs ticket system, from column M).
For each parameter the «Средние по клубам» sheet shows league average / min /
max and a per-club table with value, place (rank by the parameter's
better-direction), and a gradation (Хорошие / Удовлетворительные /
Неудовлетворительные показатели). compute_club_metrics gains price_reg and
deviation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/clubs_aggregate.xlsx
+++ b/output/clubs_aggregate.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,9 +38,15 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -49,7 +55,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="000B5CAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00E2E5EA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E4F4E4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCF4DD"/>
       </patternFill>
     </fill>
   </fills>
@@ -65,18 +86,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -442,14 +464,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:D32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,369 +490,377 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Показатель</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Среднее по клубам</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>Ед.</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>club a</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>club b</t>
-        </is>
-      </c>
+          <t>Средняя цена билета (регулярный чемпионат), руб.</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n"/>
+      <c r="C4" s="4" t="n"/>
+      <c r="D4" s="4" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Посещаемость за сезон (всего проходов)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="n">
-        <v>387093</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>чел.</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>387093</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>387093</v>
+          <t>Среднее по Лиге</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1116.5207</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Средняя посещаемость (сезон)</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="n">
-        <v>8797.5682</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>зрит./матч</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>8797.5682</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>8797.5682</v>
+          <t>Минимум</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1116.5207</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Средняя посещаемость (регулярка)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="n">
-        <v>8789.3529</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>зрит./матч</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>8789.3529</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>8789.3529</v>
+          <t>Максимум</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1116.5207</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Матчей за сезон</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="n">
-        <v>44</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>44</v>
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Платные билеты (разовые)</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="n">
-        <v>234277</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>234277</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>234277</v>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>1116.5207</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>Хорошие показатели</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Бесплатные билеты (разовые)</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>19960</v>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>19960</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>19960</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Доля бесплатных билетов</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>0.0927</v>
-      </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="n">
-        <v>0.0927</v>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>0.0927</v>
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>1116.5207</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>Удовлетворительные показатели</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Платных абонементов (продано)</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>2479</v>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>шт.</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>2479</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>2479</v>
-      </c>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Доля продаж билетов онлайн, %</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Заполняемость арены (регулярка)</t>
-        </is>
-      </c>
-      <c r="B13" s="6" t="n">
-        <v>0.9804</v>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D13" s="7" t="n">
-        <v>0.9804</v>
-      </c>
-      <c r="E13" s="7" t="n">
-        <v>0.9804</v>
+          <t>Среднее по Лиге</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>0.8476</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Доход — всего за сезон</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n">
-        <v>510511394.8</v>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="n">
-        <v>510511394.8</v>
-      </c>
-      <c r="E14" s="5" t="n">
-        <v>510511394.8</v>
+          <t>Минимум</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.8476</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Доход от платных билетов</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="n">
-        <v>379145691.8</v>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>379145691.8</v>
-      </c>
-      <c r="E15" s="5" t="n">
-        <v>379145691.8</v>
+          <t>Максимум</t>
+        </is>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>0.8476</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Доход от абонементов</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="n">
-        <v>78873675</v>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="n">
-        <v>78873675</v>
-      </c>
-      <c r="E16" s="5" t="n">
-        <v>78873675</v>
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Средняя цена платного билета (сезон)</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="n">
-        <v>1618.365</v>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>1618.365</v>
-      </c>
-      <c r="E17" s="5" t="n">
-        <v>1618.365</v>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>0.8476</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>Хорошие показатели</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Стоимость абонемента (сезон)</t>
-        </is>
-      </c>
-      <c r="B18" s="4" t="n">
-        <v>31816.7305</v>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>руб.</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="n">
-        <v>31816.7305</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>31816.7305</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Доля онлайн-продаж</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="n">
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="n">
         <v>0.8476</v>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D19" s="7" t="n">
-        <v>0.8476</v>
-      </c>
-      <c r="E19" s="7" t="n">
-        <v>0.8476</v>
+      <c r="C18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>Удовлетворительные показатели</t>
+        </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Агентская комиссия (средняя)</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Доля бесплатных билетов, %</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="n"/>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Среднее по Лиге</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n">
+        <v>0.0927</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Минимум</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="n">
+        <v>0.0927</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Максимум</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>0.0927</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="8" t="inlineStr">
+        <is>
+          <t>Хорошие показатели</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B26" s="11" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>Удовлетворительные показатели</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Фактическое отклонение посещаемости, %</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="n"/>
+      <c r="D28" s="4" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Нет данных по параметру</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Aggregate: add total revenue and agent commission parameters
Extend the club aggregate PARAMS with «Общая выручка (за сезон)» (higher is
better) and «Агентская комиссия (средняя)» (lower is better). Both flow into
the xlsx and docx aggregates with league avg/min/max, per-club place, and
gradation.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013rLJ6hxzv9KFUkktTn1LMi
</commit_message>
<xml_diff>
--- a/output/clubs_aggregate.xlsx
+++ b/output/clubs_aggregate.xlsx
@@ -464,7 +464,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -588,7 +588,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Доля продаж билетов онлайн, %</t>
+          <t>Общая выручка (за сезон), руб.</t>
         </is>
       </c>
       <c r="B12" s="4" t="n"/>
@@ -601,8 +601,8 @@
           <t>Среднее по Лиге</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n">
-        <v>0.8476</v>
+      <c r="B13" s="5" t="n">
+        <v>510511394.8</v>
       </c>
     </row>
     <row r="14">
@@ -611,8 +611,8 @@
           <t>Минимум</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
-        <v>0.8476</v>
+      <c r="B14" s="5" t="n">
+        <v>510511394.8</v>
       </c>
     </row>
     <row r="15">
@@ -621,8 +621,8 @@
           <t>Максимум</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
-        <v>0.8476</v>
+      <c r="B15" s="5" t="n">
+        <v>510511394.8</v>
       </c>
     </row>
     <row r="16">
@@ -653,8 +653,8 @@
           <t>club a</t>
         </is>
       </c>
-      <c r="B17" s="11" t="n">
-        <v>0.8476</v>
+      <c r="B17" s="7" t="n">
+        <v>510511394.8</v>
       </c>
       <c r="C17" s="2" t="n">
         <v>1</v>
@@ -671,8 +671,8 @@
           <t>club b</t>
         </is>
       </c>
-      <c r="B18" s="11" t="n">
-        <v>0.8476</v>
+      <c r="B18" s="7" t="n">
+        <v>510511394.8</v>
       </c>
       <c r="C18" s="2" t="n">
         <v>2</v>
@@ -686,7 +686,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Доля бесплатных билетов, %</t>
+          <t>Доля продаж билетов онлайн, %</t>
         </is>
       </c>
       <c r="B20" s="4" t="n"/>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B21" s="10" t="n">
-        <v>0.0927</v>
+        <v>0.8476</v>
       </c>
     </row>
     <row r="22">
@@ -710,7 +710,7 @@
         </is>
       </c>
       <c r="B22" s="10" t="n">
-        <v>0.0927</v>
+        <v>0.8476</v>
       </c>
     </row>
     <row r="23">
@@ -720,7 +720,7 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>0.0927</v>
+        <v>0.8476</v>
       </c>
     </row>
     <row r="24">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B25" s="11" t="n">
-        <v>0.0927</v>
+        <v>0.8476</v>
       </c>
       <c r="C25" s="2" t="n">
         <v>1</v>
@@ -770,7 +770,7 @@
         </is>
       </c>
       <c r="B26" s="11" t="n">
-        <v>0.0927</v>
+        <v>0.8476</v>
       </c>
       <c r="C26" s="2" t="n">
         <v>2</v>
@@ -784,7 +784,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>Фактическое отклонение посещаемости, %</t>
+          <t>Доля бесплатных билетов, %</t>
         </is>
       </c>
       <c r="B28" s="4" t="n"/>
@@ -794,71 +794,252 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Нет данных по параметру</t>
-        </is>
+          <t>Среднее по Лиге</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>0.0927</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="6" t="inlineStr">
-        <is>
-          <t>Клуб</t>
-        </is>
-      </c>
-      <c r="B30" s="6" t="inlineStr">
-        <is>
-          <t>Значение</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Место</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="inlineStr">
-        <is>
-          <t>Градация</t>
-        </is>
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Минимум</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>0.0927</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
+          <t>Максимум</t>
+        </is>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>0.0927</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
           <t>club a</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B33" s="11" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="C33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="8" t="inlineStr">
+        <is>
+          <t>Хорошие показатели</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="n">
+        <v>0.0927</v>
+      </c>
+      <c r="C34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D34" s="9" t="inlineStr">
+        <is>
+          <t>Удовлетворительные показатели</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Агентская комиссия (средняя), %</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="n"/>
+      <c r="C36" s="4" t="n"/>
+      <c r="D36" s="4" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Нет данных по параметру</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>нет данных</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
         <is>
           <t>club b</t>
         </is>
       </c>
-      <c r="B32" s="2" t="inlineStr">
+      <c r="B40" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C32" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D32" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Фактическое отклонение посещаемости, %</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="n"/>
+      <c r="C42" s="4" t="n"/>
+      <c r="D42" s="4" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>Нет данных по параметру</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Клуб</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
+          <t>Значение</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>Место</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="inlineStr">
+        <is>
+          <t>Градация</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>club a</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>нет данных</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>club b</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>нет данных</t>
         </is>

</xml_diff>